<commit_message>
Yangın yükü modülü (bölüm bazında), Tanyeri-Tuzla projesi ve varsayım listesi
- q = Σ(kütle × alt ısıl değer)/alan, odun eşdeğeri, bölüm alanı Ek-4 (üretim/depo) kontrolü
- Masaüstü 'Yangın yükü' sekmesi, form tabloları (T7/T8), hesap dökümü ve raporlar
- Tanyeri (Tuzla) projesi: mahal listesi, kompartıman malzemeleri, varsayımlar ve açık sorular

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y65w22BhwpQqtFCs8yHq45
</commit_message>
<xml_diff>
--- a/belgeler/Isveren_Veri_Toplama_Formu.xlsx
+++ b/belgeler/Isveren_Veri_Toplama_Formu.xlsx
@@ -20,10 +20,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3_Merdivenler" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4_Kapilar" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5_Duman_Mahalleri" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T6_Yanici_Sivi" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Belgeler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notlar" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listeler" sheetId="17" state="hidden" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T7_Yangin_Yuku_Bolumleri" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T8_Yangin_Yuku_Malzeme" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T6_Yanici_Sivi" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Belgeler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notlar" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listeler" sheetId="19" state="hidden" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C28"/>
+  <dimension ref="B1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -839,34 +841,58 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>T6_Yanici_Sivi</t>
+          <t>T7_Yangin_Yuku_Bolumleri</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Tablo 6 — Yanıcı / parlayıcı sıvı tankları ve depolama</t>
+          <t>Tablo 7 — Yangın yükü: bölümler (kompartımanlar)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Belgeler</t>
+          <t>T8_Yangin_Yuku_Malzeme</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>İşletmeden istenecek belge kontrol listesi</t>
+          <t>Tablo 8 — Yangın yükü: bölümlerdeki yanıcı malzemeler</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
+          <t>T6_Yanici_Sivi</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tablo 6 — Yanıcı / parlayıcı sıvı tankları ve depolama</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Belgeler</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>İşletmeden istenecek belge kontrol listesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Notlar</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Forma sığmayan ek bilgiler</t>
         </is>
@@ -3401,6 +3427,719 @@
   <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="30.76923076923077" customWidth="1" min="1" max="1"/>
+    <col width="15.38461538461539" customWidth="1" min="2" max="2"/>
+    <col width="18.46153846153846" customWidth="1" min="3" max="3"/>
+    <col width="23.07692307692308" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Tablo 7 — Yangın yükü: bölümler (kompartımanlar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Yangın duvarlarıyla ayrılmış (veya ayrılması planlanan) her bölüm/kompartıman için bir satır: adı ve alanı.   [Kim: İŞVEREN — varsa / biliyorsa.  Kaynak: Mimari plan, kompartıman çalışması]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Satır 6 örnektir (programa aktarılmaz). Verilerinizi 7. satırdan itibaren yazın.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Bölüm / kompartıman</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Alan (m²)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Kat</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Kullanım</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Bölümün adı (ör. Depo alt, Boyahane, Montaj). Tablo 8'deki bölüm adıyla AYNI yazın.</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Bölümün alanı (m²) — mimari plandan.</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Bulunduğu kat (bilgi).</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Bölüm üretim alanı ise 'Endüstriyel (üretim)', depo ise 'Depo' seçin (Ek-4 kompartıman sınırı buna göre değişir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>ÖRN: Depo alt</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>974.1799999999999</v>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>1. kat</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Depo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="n"/>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="n"/>
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="18" t="n"/>
+      <c r="D14" s="18" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="18" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="n"/>
+      <c r="B34" s="18" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="18" t="n"/>
+      <c r="C35" s="18" t="n"/>
+      <c r="D35" s="18" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="n"/>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="18" t="n"/>
+      <c r="D36" s="18" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="18" t="n"/>
+      <c r="C37" s="18" t="n"/>
+      <c r="D37" s="18" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="n"/>
+      <c r="B38" s="18" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="n"/>
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="n"/>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="n"/>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="18" t="n"/>
+      <c r="D44" s="18" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="n"/>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B7:B46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen 0 veya daha büyük bir sayı yazın." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="D7:D46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Lütfen açılır listeden seçin." type="list">
+      <formula1>=Listeler!$P$1:$P$2</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30.76923076923077" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="15.38461538461539" customWidth="1" min="3" max="3"/>
+    <col width="27.69230769230769" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Tablo 8 — Yangın yükü: bölümlerdeki yanıcı malzemeler</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Her bölümde bulunan yanıcı malzeme türü ve ortalama/azami miktarı (kg). Aynı bölümde birden fazla malzeme için ayrı satır yazın.   [Kim: İŞVEREN — varsa / biliyorsa.  Kaynak: Depo/üretim stok kayıtları, ambalaj ve malzeme listeleri, MSDS]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Satır 6 örnektir (programa aktarılmaz). Verilerinizi 7. satırdan itibaren yazın.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Bölüm / kompartıman</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Malzeme</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Miktar (kg)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Isıl değer (MJ/kg) [0=tablodan]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Tablo 7'deki bölüm adı.</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Malzeme türünü listeden seçin (alt ısıl değeri otomatik gelir).</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Bölümde bulunan miktar (kg). Dolu koli/kasa için içindekiler dahil toplam kütle.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>MSDS veya laboratuvar ısıl değeri (MJ/kg) biliniyorsa yazın; boşsa listedeki ortalama değer kullanılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>ÖRN: Depo alt</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Ahşap (palet, kereste, kontrplak)</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" s="17" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="n"/>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="n"/>
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="18" t="n"/>
+      <c r="D14" s="18" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="18" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="n"/>
+      <c r="B34" s="18" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="18" t="n"/>
+      <c r="C35" s="18" t="n"/>
+      <c r="D35" s="18" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="n"/>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="18" t="n"/>
+      <c r="D36" s="18" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="18" t="n"/>
+      <c r="C37" s="18" t="n"/>
+      <c r="D37" s="18" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="n"/>
+      <c r="B38" s="18" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="n"/>
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="n"/>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="n"/>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="18" t="n"/>
+      <c r="D44" s="18" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="n"/>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B7:B46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Lütfen açılır listeden seçin." type="list">
+      <formula1>=Listeler!$Q$1:$Q$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7:C46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen 0 veya daha büyük bir sayı yazın." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="D7:D46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen 0 veya daha büyük bir sayı yazın." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
     <col width="24.61538461538462" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15.38461538461539" customWidth="1" min="3" max="3"/>
@@ -3738,13 +4477,13 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B7:B46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Lütfen açılır listeden seçin." type="list">
-      <formula1>=Listeler!$P$1:$P$6</formula1>
+      <formula1>=Listeler!$R$1:$R$6</formula1>
     </dataValidation>
     <dataValidation sqref="C7:C46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz değer" error="Lütfen 0 veya daha büyük bir sayı yazın." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="D7:D46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz seçim" error="Lütfen açılır listeden seçin." type="list">
-      <formula1>=Listeler!$Q$1:$Q$3</formula1>
+      <formula1>=Listeler!$S$1:$S$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3752,7 +4491,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4293,7 +5032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4387,13 +5126,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:S42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4474,10 +5213,20 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>Endüstriyel (üretim)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Ahşap (palet, kereste, kontrplak)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>yerustu</t>
         </is>
@@ -4561,10 +5310,20 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>Depo</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Karton / kâğıt (koli, ambalaj)</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>IB</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>yeralti</t>
         </is>
@@ -4616,12 +5375,17 @@
           <t>bodrum_depo</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Plastik — PE / PP (kasa, mamül)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>depo_icinde</t>
         </is>
@@ -4673,7 +5437,12 @@
           <t>diger</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Plastik — PS (polistiren)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>II</t>
         </is>
@@ -4705,7 +5474,12 @@
           <t>Ofis, dernek merkezi, halk kütüphanesi</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Plastik — ABS</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>IIIA</t>
         </is>
@@ -4732,7 +5506,12 @@
           <t>Yemekhane / kantin / lokanta (net alan)</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Plastik — PVC</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>IIIB</t>
         </is>
@@ -4759,6 +5538,11 @@
           <t>Toplantı, konferans, çok amaçlı salon (net alan)</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Plastik — PA (naylon) / polyester</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4781,6 +5565,11 @@
           <t>Derslik, bilgisayar odası, seminer salonu</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Kauçuk / lastik</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4803,6 +5592,11 @@
           <t>Resepsiyon, bekleme alanı, atrium zemini</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Tekstil (pamuk, elyaf)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4820,6 +5614,11 @@
           <t>Süpermarket, mağaza, dükkân</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Mineral yağ / gres</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -4832,6 +5631,11 @@
           <t>Sanat galerisi, müze</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Solvent bazlı sıvı boya / vernik (varsayım)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -4844,6 +5648,11 @@
           <t>Sergi alanı, stüdyo (net alan)</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Tiner / solvent (varsayım)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -4854,6 +5663,11 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>Terminal bekleme salonu (net alan)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Diğer (ısıl değeri elle gir)</t>
         </is>
       </c>
     </row>

</xml_diff>